<commit_message>
Entretien cotisations du 19/10/2026 : compte rendu, note interne, PBC complémentaire, guides, rapport v4 avec logigrammes
- Compte rendu d'entretien (12 diapositives) avec circuit des précomptes et parcours des recrues en logigrammes
- Note interne confidentielle sur l'entretien cotisations
- PBC complémentaire cotisations (items 56 à 70, fichiers manquants, modèles de données) reportée dans la PBC générale
- Guides : réponses et relances (onglet 4), questions 24 à 27 rétablies et section H (onglet 2)
- Rapport v4 et classeur v4 : chaîne de traitement, circuit des précomptes et nouvelles recrues en logigrammes modifiables

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QrZoDwZJKb9thfUp96Ro9x
</commit_message>
<xml_diff>
--- a/FPPN_Guides_entretiens_actuariat_20261019.xlsx
+++ b/FPPN_Guides_entretiens_actuariat_20261019.xlsx
@@ -2477,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:L50"/>
+  <dimension ref="B2:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -3719,8 +3719,8 @@
           <t>Attendu : rapport d'étude et accusé de dépôt, ou non. Si non, la présente mission peut y contribuer.</t>
         </is>
       </c>
-      <c r="G38" s="6" t="inlineStr"/>
-      <c r="H38" s="6" t="inlineStr"/>
+      <c r="G38" s="6" t="n"/>
+      <c r="H38" s="6" t="n"/>
       <c r="I38" s="6" t="inlineStr">
         <is>
           <t>Règlement d'exécution n° 004/2022/COM/UEMOA, art. 14</t>
@@ -3764,8 +3764,8 @@
           <t>Attendu : rapports du commissaire aux comptes 2020 à 2025 ; états par risque long.</t>
         </is>
       </c>
-      <c r="G39" s="6" t="inlineStr"/>
-      <c r="H39" s="6" t="inlineStr"/>
+      <c r="G39" s="6" t="n"/>
+      <c r="H39" s="6" t="n"/>
       <c r="I39" s="6" t="inlineStr">
         <is>
           <t>Règlement d'exécution n° 004/2022/COM/UEMOA, art. 12, 13 et 15</t>
@@ -3862,8 +3862,8 @@
           <t>Attendu : une décision ou une recommandation du commissaire aux comptes. Sinon, reclasser en compte 190.</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr"/>
-      <c r="H41" s="6" t="inlineStr"/>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="6" t="n"/>
       <c r="I41" s="6" t="inlineStr">
         <is>
           <t>PCMS, liste des comptes et fiche n° 6</t>
@@ -4036,59 +4036,166 @@
       </c>
       <c r="L44" s="6" t="n"/>
     </row>
-    <row r="45"/>
-    <row r="46">
-      <c r="B46" s="2" t="inlineStr">
+    <row r="45">
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>H. Cotisations : questions issues de l'entretien du 19/10/2026 (chef comptable)</t>
+        </is>
+      </c>
+      <c r="C45" s="15" t="n"/>
+      <c r="D45" s="15" t="n"/>
+      <c r="E45" s="15" t="n"/>
+      <c r="F45" s="15" t="n"/>
+      <c r="G45" s="15" t="n"/>
+      <c r="H45" s="15" t="n"/>
+      <c r="I45" s="15" t="n"/>
+      <c r="J45" s="15" t="n"/>
+      <c r="K45" s="15" t="n"/>
+      <c r="L45" s="16" t="n"/>
+    </row>
+    <row r="46" ht="46" customHeight="1">
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Cotisations</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>Comment les paiements manuels de cotisations sont-ils encaissés, comptabilisés et suivis ?</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>Mesurer les cotisations qui échappent aux fichiers de précomptes.</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>Le responsable des cotisations indique que des paiements manuels sont possibles et enregistrés avec date et heure (entretien du 19/10/2026). Attendu : compte d'encaissement, état des paiements.</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="n"/>
+      <c r="H46" s="6" t="n"/>
+      <c r="I46" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J46" s="6" t="inlineStr">
+        <is>
+          <t>Liste des paiements manuels (PBC, item 65)</t>
+        </is>
+      </c>
+      <c r="K46" s="6" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L46" s="6" t="n"/>
+    </row>
+    <row r="47" ht="46" customHeight="1">
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Cotisations</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Quelle est la clé de répartition du taux de cotisation entre maladie (poste 936) et décès (poste 8Z6) ?</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>Le responsable des cotisations renvoie cette répartition à la comptabilité.</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>Les fichiers retour montrent 3,77 % et 1,23 % du salaire de base. Attendu : la clé et le texte qui la fixe.</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="n"/>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>Taux maladie + taux décès = 5,00 % du salaire de base (fichiers retour)</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J47" s="6" t="inlineStr">
+        <is>
+          <t>Barème (PBC, item 56)</t>
+        </is>
+      </c>
+      <c r="K47" s="6" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L47" s="6" t="n"/>
+    </row>
+    <row r="49">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>Clôture de l'entretien</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="18" t="inlineStr">
-        <is>
-          <t>•  Récapituler les documents à obtenir : détail et fichiers de calcul des provisions 2019-2026, rapport actuariel existant, courriers de l'AIRMS, description de l'épargne et taux servis.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="18" t="inlineStr">
-        <is>
-          <t>•  Demander : « Qui d'autre dois-je voir sur ces sujets ? »</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="B49" s="18" t="inlineStr">
-        <is>
-          <t>•  Convenir d'une date de remise des documents et d'un contact pour les questions de suivi.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="18" t="inlineStr">
         <is>
+          <t>•  Récapituler les documents à obtenir : détail et fichiers de calcul des provisions 2019-2026, rapport actuariel existant, courriers de l'AIRMS, description de l'épargne et taux servis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="18" t="inlineStr">
+        <is>
+          <t>•  Demander : « Qui d'autre dois-je voir sur ces sujets ? »</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>•  Convenir d'une date de remise des documents et d'un contact pour les questions de suivi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="18" t="inlineStr">
+        <is>
           <t>•  Remercier l'interlocuteur.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="9">
     <mergeCell ref="B4:L4"/>
-    <mergeCell ref="B41:L41"/>
     <mergeCell ref="B30:L30"/>
-    <mergeCell ref="B38:L38"/>
     <mergeCell ref="B33:L33"/>
-    <mergeCell ref="B39:L39"/>
     <mergeCell ref="B23:L23"/>
-    <mergeCell ref="B40:L40"/>
     <mergeCell ref="B5:L5"/>
+    <mergeCell ref="B45:L45"/>
     <mergeCell ref="B17:L17"/>
     <mergeCell ref="B27:L27"/>
     <mergeCell ref="B8:L8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="K8:K36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K8:K47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5145,7 +5252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:L39"/>
+  <dimension ref="B2:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -5172,7 +5279,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>19 octobre 2026, 10h, avec Ruth Miensa</t>
+          <t>19 octobre 2026, 10h, avec Ruth Miensa ; entretien tenu avec le responsable des cotisations, également responsable informatique (nom à compléter)</t>
         </is>
       </c>
     </row>
@@ -5301,9 +5408,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="46" customHeight="1">
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 (déclaration à confirmer par document) : maladie et décès en pourcentage du salaire de base ; autres produits en montants fixes (EFC, PEP, MEDOC, prêts, flotte). Barème à déposer sur la plateforme de partage, non reçu (PBC, item 56).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
       <c r="B10" s="5" t="n">
         <v>2</v>
       </c>
@@ -5344,9 +5455,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11" ht="46" customHeight="1">
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 (déclaration à confirmer par document) : la répartition du taux entre maladie et décès relève de la comptabilité. Question reportée au chef comptable (onglet 2, question 32).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
       <c r="B11" s="5" t="n">
         <v>3</v>
       </c>
@@ -5387,9 +5502,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr"/>
-    </row>
-    <row r="12" ht="46" customHeight="1">
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 (déclaration à confirmer par document) : fichier aller des retraités produit par le responsable des cotisations et déposé sur la plateforme de partage ; fichier retour déposé par la CGRAE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
       <c r="B12" s="5" t="n">
         <v>4</v>
       </c>
@@ -5422,7 +5541,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L12" s="6" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 (déclaration à confirmer par document) : l'EFC et le PEP sont présentés aux élèves policiers comme obligatoires dès l'école, sans texte. Délai d'au moins trois mois de cotisation avant les prestations (à recouper avec l'entretien du 16/10/2026).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="B13" s="14" t="inlineStr">
@@ -5441,7 +5564,7 @@
       <c r="K13" s="15" t="n"/>
       <c r="L13" s="16" t="n"/>
     </row>
-    <row r="14" ht="46" customHeight="1">
+    <row r="14" ht="60" customHeight="1">
       <c r="B14" s="5" t="n">
         <v>5</v>
       </c>
@@ -5474,9 +5597,13 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr"/>
-    </row>
-    <row r="15" ht="32" customHeight="1">
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 (déclaration à confirmer par document) : précompte sur salaire. Maladie et décès : fichier aller transmis directement par la direction du personnel de la Police à la Solde, sans plateforme de partage ; retour reçu en direct par le FPPN, canal à préciser. Produits complémentaires, CGRAE et GNA : fichiers aller produits et déposés sur la plateforme de partage par le responsable des cotisations, retours déposés par l'entité concernée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
       <c r="B15" s="5" t="n">
         <v>6</v>
       </c>
@@ -5517,9 +5644,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr"/>
-    </row>
-    <row r="16" ht="46" customHeight="1">
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
       <c r="B16" s="5" t="n">
         <v>7</v>
       </c>
@@ -5564,7 +5695,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr"/>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="B17" s="14" t="inlineStr">
@@ -5583,7 +5718,7 @@
       <c r="K17" s="15" t="n"/>
       <c r="L17" s="16" t="n"/>
     </row>
-    <row r="18" ht="32" customHeight="1">
+    <row r="18" ht="60" customHeight="1">
       <c r="B18" s="5" t="n">
         <v>8</v>
       </c>
@@ -5616,7 +5751,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L18" s="6" t="inlineStr"/>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="B19" s="5" t="n">
@@ -5663,9 +5802,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20" ht="46" customHeight="1">
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 (déclaration à confirmer par document) : le fichier aller contient le mécano, le nom, le code du poste, une référence et le montant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1">
       <c r="B20" s="5" t="n">
         <v>10</v>
       </c>
@@ -5698,9 +5841,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21" ht="46" customHeight="1">
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 (déclaration à confirmer par document) : les élèves policiers souscrivent avec leur seul matricule ; le mécano est reporté en masse sur les fiches après son attribution, et le premier précompte peut être décalé d'un mois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="60" customHeight="1">
       <c r="B21" s="5" t="n">
         <v>11</v>
       </c>
@@ -5741,9 +5888,13 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L21" s="6" t="inlineStr"/>
-    </row>
-    <row r="22" ht="46" customHeight="1">
+      <c r="L21" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 (déclaration à confirmer par document) : aucun rapprochement entre fichiers aller et retour, aucun état des cotisations, aucun suivi mutualiste par mutualiste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1">
       <c r="B22" s="5" t="n">
         <v>12</v>
       </c>
@@ -5788,9 +5939,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23" ht="46" customHeight="1">
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1">
       <c r="B23" s="5" t="n">
         <v>13</v>
       </c>
@@ -5827,9 +5982,13 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L23" s="6" t="inlineStr"/>
-    </row>
-    <row r="24" ht="32" customHeight="1">
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 (déclaration à confirmer par document) : fichier des ayants droit attendu, sans les âges (PBC, item 66).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1">
       <c r="B24" s="5" t="n">
         <v>14</v>
       </c>
@@ -5874,7 +6033,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L24" s="6" t="inlineStr"/>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="14" t="inlineStr">
@@ -5893,7 +6056,7 @@
       <c r="K25" s="15" t="n"/>
       <c r="L25" s="16" t="n"/>
     </row>
-    <row r="26" ht="32" customHeight="1">
+    <row r="26" ht="60" customHeight="1">
       <c r="B26" s="5" t="n">
         <v>15</v>
       </c>
@@ -5926,9 +6089,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L26" s="6" t="inlineStr"/>
-    </row>
-    <row r="27" ht="46" customHeight="1">
+      <c r="L26" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 (déclaration à confirmer par document) : EFC : 6 000 FCFA avant 2021, 10 000 FCFA pour les nouvelles souscriptions depuis 2021 ; les anciens restent à 6 000 FCFA mais peuvent passer à 10 000 FCFA ; aucun document formel. PEP : à partir de 10 000 FCFA, par paliers de 5 000 FCFA ; durée à vérifier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="60" customHeight="1">
       <c r="B27" s="5" t="n">
         <v>16</v>
       </c>
@@ -5973,7 +6140,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L27" s="6" t="inlineStr"/>
+      <c r="L27" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="B28" s="14" t="inlineStr">
@@ -5992,7 +6163,7 @@
       <c r="K28" s="15" t="n"/>
       <c r="L28" s="16" t="n"/>
     </row>
-    <row r="29" ht="32" customHeight="1">
+    <row r="29" ht="60" customHeight="1">
       <c r="B29" s="5" t="n">
         <v>17</v>
       </c>
@@ -6025,9 +6196,13 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L29" s="6" t="inlineStr"/>
-    </row>
-    <row r="30" ht="32" customHeight="1">
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 (déclaration à confirmer par document) : aucun contrôle des retours. Un état séparé des motifs de rejet n'est reçu que depuis environ deux mois. Paiements manuels possibles, enregistrés avec date et heure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="60" customHeight="1">
       <c r="B30" s="5" t="n">
         <v>18</v>
       </c>
@@ -6068,7 +6243,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L30" s="6" t="inlineStr"/>
+      <c r="L30" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 (déclaration à confirmer par document) : aucun suivi des écarts entre cotisations demandées et précomptées.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="14" t="inlineStr">
@@ -6087,7 +6266,7 @@
       <c r="K31" s="15" t="n"/>
       <c r="L31" s="16" t="n"/>
     </row>
-    <row r="32" ht="32" customHeight="1">
+    <row r="32" ht="60" customHeight="1">
       <c r="B32" s="5" t="n">
         <v>19</v>
       </c>
@@ -6120,9 +6299,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L32" s="6" t="inlineStr"/>
-    </row>
-    <row r="33" ht="46" customHeight="1">
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 (déclaration à confirmer par document) : l'interlocuteur est le responsable informatique ; il gère les cotisations parce qu'il maîtrise le logiciel qui produit les fichiers. Nom du logiciel non relevé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="60" customHeight="1">
       <c r="B33" s="5" t="n">
         <v>20</v>
       </c>
@@ -6167,60 +6350,442 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L33" s="6" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="B35" s="2" t="inlineStr">
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>G. Relances après l'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="C34" s="15" t="n"/>
+      <c r="D34" s="15" t="n"/>
+      <c r="E34" s="15" t="n"/>
+      <c r="F34" s="15" t="n"/>
+      <c r="G34" s="15" t="n"/>
+      <c r="H34" s="15" t="n"/>
+      <c r="I34" s="15" t="n"/>
+      <c r="J34" s="15" t="n"/>
+      <c r="K34" s="15" t="n"/>
+      <c r="L34" s="16" t="n"/>
+    </row>
+    <row r="35" ht="46" customHeight="1">
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Circuit</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Par quel canal le FPPN reçoit-il les fichiers retour maladie (936) et décès (8Z6), et qui les reçoit ?</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Compléter le circuit des précomptes obligatoires.</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : courriel, support physique ou dépôt par la Solde, avec le nom du destinataire au FPPN.</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="n"/>
+      <c r="H35" s="6" t="n"/>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>Fichiers retour manquants (PBC, item 62)</t>
+        </is>
+      </c>
+      <c r="K35" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="n"/>
+    </row>
+    <row r="36" ht="46" customHeight="1">
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Rejets</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Depuis quelle date exacte la Solde transmet-elle l'état des motifs de rejet ?</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Savoir à partir de quel mois les écarts peuvent être expliqués.</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : une date et les états reçus. L'interlocuteur cite environ deux mois.</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="n"/>
+      <c r="H36" s="6" t="n"/>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>États des motifs de rejet (PBC, item 64)</t>
+        </is>
+      </c>
+      <c r="K36" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L36" s="6" t="n"/>
+    </row>
+    <row r="37" ht="46" customHeight="1">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Quelle est la durée d'un plan PEP et quelles sont les conditions de retrait ?</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Établir l'échéancier de l'épargne.</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : règlement du PEP. La durée n'a pas été précisée le 19/10/2026.</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="n"/>
+      <c r="H37" s="6" t="n"/>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>Documentation des produits (PBC, item 57)</t>
+        </is>
+      </c>
+      <c r="K37" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="n"/>
+    </row>
+    <row r="38" ht="46" customHeight="1">
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Prestations</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Le délai d'au moins trois mois de cotisation s'applique-t-il à tous les produits, y compris la maladie et le décès ? Quel texte le fixe ?</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Lever la contradiction avec l'entretien du 16/10/2026, qui indiquait l'absence de délai de carence pour le régime obligatoire.</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : un texte et la liste des produits concernés.</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="n"/>
+      <c r="H38" s="6" t="n"/>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026 ; compte rendu du 16/10/2026</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>Règle des trois mois (PBC, item 59)</t>
+        </is>
+      </c>
+      <c r="K38" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L38" s="6" t="n"/>
+    </row>
+    <row r="39" ht="46" customHeight="1">
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Grenier</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Quels sont les types de prêts du Grenier et leurs conditions ?</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Rapprocher les trois types cités des huit types de crédit présents dans les fichiers de production.</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : liste des types de prêts, montants, durées, taux.</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="n"/>
+      <c r="H39" s="6" t="n"/>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026 ; fichiers de production du Grenier reçus le 15/10/2026</t>
+        </is>
+      </c>
+      <c r="J39" s="6" t="inlineStr">
+        <is>
+          <t>Types de prêts (PBC, item 70)</t>
+        </is>
+      </c>
+      <c r="K39" s="17" t="inlineStr">
+        <is>
+          <t>Si le temps le permet</t>
+        </is>
+      </c>
+      <c r="L39" s="6" t="n"/>
+    </row>
+    <row r="40" ht="46" customHeight="1">
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>MEDOC</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Sur quelle période MEDOC a-t-il fonctionné, et quand a-t-il été suspendu ?</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Expliquer les mois sans fichier du poste 8Z7.</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : date de démarrage, date de suspension, conventions avec les pharmacies.</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="n"/>
+      <c r="H40" s="6" t="n"/>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>Documentation MEDOC (PBC, item 69)</t>
+        </is>
+      </c>
+      <c r="K40" s="17" t="inlineStr">
+        <is>
+          <t>Si le temps le permet</t>
+        </is>
+      </c>
+      <c r="L40" s="6" t="n"/>
+    </row>
+    <row r="41" ht="46" customHeight="1">
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Barème</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Quel document notifie à la Solde les taux maladie et décès appliqués ?</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Valider la répartition 3,77 % et 1,23 % mesurée dans les fichiers retour.</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : note ou courrier de notification des taux à la Solde.</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="6" t="n"/>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J41" s="6" t="inlineStr">
+        <is>
+          <t>Barème et notification (PBC, item 56)</t>
+        </is>
+      </c>
+      <c r="K41" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L41" s="6" t="n"/>
+    </row>
+    <row r="42" ht="46" customHeight="1">
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>Produits</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>À quelle date chaque produit a-t-il démarré : EFC, PEP, MEDOC, prêts du Grenier, flotte automobile, retraités ?</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Distinguer les mois sans fichier des mois où le produit n'existait pas.</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : une date par produit.</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="n"/>
+      <c r="H42" s="6" t="n"/>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J42" s="6" t="inlineStr">
+        <is>
+          <t>Dates de démarrage (PBC, item 60)</t>
+        </is>
+      </c>
+      <c r="K42" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L42" s="6" t="n"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Clôture de l'entretien</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="30" customHeight="1">
-      <c r="B36" s="18" t="inlineStr">
+    <row r="45" ht="30" customHeight="1">
+      <c r="B45" s="18" t="inlineStr">
         <is>
           <t>•  Récapituler les documents à obtenir : barème des cotisations 2020-2026, fichiers des mutualistes et des ayants droit 2019-2026, état des cotisations non reversées, mouvements d'effectifs.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="B37" s="18" t="inlineStr">
+    <row r="46" ht="16" customHeight="1">
+      <c r="B46" s="18" t="inlineStr">
         <is>
           <t>•  Demander : « Qui d'autre dois-je voir sur ces sujets ? »</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="B38" s="18" t="inlineStr">
+    <row r="47" ht="16" customHeight="1">
+      <c r="B47" s="18" t="inlineStr">
         <is>
           <t>•  Convenir d'une date de remise des documents et d'un contact pour les questions de suivi.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="B39" s="18" t="inlineStr">
+    <row r="48" ht="16" customHeight="1">
+      <c r="B48" s="18" t="inlineStr">
         <is>
           <t>•  Remercier l'interlocuteur.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="B4:L4"/>
     <mergeCell ref="B13:L13"/>
-    <mergeCell ref="B38:L38"/>
-    <mergeCell ref="B39:L39"/>
+    <mergeCell ref="B48:L48"/>
     <mergeCell ref="B25:L25"/>
+    <mergeCell ref="B47:L47"/>
     <mergeCell ref="B5:L5"/>
-    <mergeCell ref="B37:L37"/>
+    <mergeCell ref="B34:L34"/>
     <mergeCell ref="B28:L28"/>
-    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="B46:L46"/>
+    <mergeCell ref="B45:L45"/>
     <mergeCell ref="B31:L31"/>
     <mergeCell ref="B17:L17"/>
     <mergeCell ref="B8:L8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="K8:K34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K8:K43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7160,7 +7725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:M33"/>
+  <dimension ref="B2:M33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>

</xml_diff>

<commit_message>
Rapport v5 : revue des provisions, choix des formules et tableau des formules
- Revue des provisions par produit (règlement d'exécution n° 004/2022, art. 7 à 11) : PSAP et dettes envers les
  cliniques, méthode CIMA des sinistres tardifs, dépréciation des prêts du Grenier, flotte GNA, départ à la retraite
- Choix de la formule : sinistralité et frais de gestion, formule du texte et méthode du FPPN (rouge si non communiquée)
- Registre de 74 formules (annexe du rapport, onglet 11_formules du classeur v5)
- PBC générale : items 71 à 79 ; guide du chef comptable : section I

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QrZoDwZJKb9thfUp96Ro9x
</commit_message>
<xml_diff>
--- a/FPPN_Guides_entretiens_actuariat_20261019.xlsx
+++ b/FPPN_Guides_entretiens_actuariat_20261019.xlsx
@@ -2477,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:L53"/>
+  <dimension ref="A2:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -4147,45 +4147,362 @@
       </c>
       <c r="L47" s="6" t="n"/>
     </row>
-    <row r="49">
-      <c r="B49" s="2" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>I. Provisions et engagements (revue du rapport v5, 19/10/2026)</t>
+        </is>
+      </c>
+      <c r="C48" s="15" t="n"/>
+      <c r="D48" s="15" t="n"/>
+      <c r="E48" s="15" t="n"/>
+      <c r="F48" s="15" t="n"/>
+      <c r="G48" s="15" t="n"/>
+      <c r="H48" s="15" t="n"/>
+      <c r="I48" s="15" t="n"/>
+      <c r="J48" s="15" t="n"/>
+      <c r="K48" s="15" t="n"/>
+      <c r="L48" s="16" t="n"/>
+    </row>
+    <row r="49" ht="46" customHeight="1">
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>Provisions</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Comment les provisions maladie et obsèques ont-elles été calculées, et pourquoi n'ont-elles pas changé depuis 2020 ?</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>Les montants sont identiques au franc près de 2020 au 31/08/2026.</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : note de calcul, liste des dossiers. Alerte : aucun calcul, montant hérité.</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>Dossier par dossier, puis sinistres tardifs (méthode CIMA)</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>PSAP = dossiers connus + tardifs</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>Règlement d'exécution n° 004/2022/COM/UEMOA, art. 10</t>
+        </is>
+      </c>
+      <c r="J49" s="6" t="inlineStr">
+        <is>
+          <t>Note de calcul (PBC, item 72)</t>
+        </is>
+      </c>
+      <c r="K49" s="6" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L49" s="6" t="n"/>
+    </row>
+    <row r="50" ht="46" customHeight="1">
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>Provisions</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>Les factures des cliniques enregistrées en dettes (compte 40110000) sont-elles aussi comprises dans la provision maladie ?</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>Éviter un double compte entre dettes et provision.</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : non, la provision couvre les soins non encore facturés.</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="n"/>
+      <c r="H50" s="6" t="n"/>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>Règlement d'exécution n° 004/2022, art. 10 ; PCMS</t>
+        </is>
+      </c>
+      <c r="J50" s="6" t="n"/>
+      <c r="K50" s="6" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L50" s="6" t="n"/>
+    </row>
+    <row r="51" ht="46" customHeight="1">
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>Grenier</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Le FPPN déprécie-t-il les prêts du Grenier en retard ? Selon quels taux ?</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>Aucune dépréciation passée depuis 2022 alors que des prêts ont plus d'un an de retard.</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : politique écrite. Sinon, barème BCEAO des SFD en référence.</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>Encours par tranche × taux</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>Dépréciation = Σ encours(k) × taux(k)</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>PCMS, principe de prudence ; BCEAO (SFD)</t>
+        </is>
+      </c>
+      <c r="J51" s="6" t="inlineStr">
+        <is>
+          <t>Politique de dépréciation (PBC, item 73)</t>
+        </is>
+      </c>
+      <c r="K51" s="6" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L51" s="6" t="n"/>
+    </row>
+    <row r="52" ht="46" customHeight="1">
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>Flotte automobile</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>Quelle est la nature des mouvements du compte 47111106 « GNA ASSURANCE » ?</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>Les primes iraient directement à GNA, mais le compte est mouvementé depuis 2023.</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : avances, remboursements de trop-perçus ou primes.</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="n"/>
+      <c r="H52" s="6" t="n"/>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>Convention avec GNA</t>
+        </is>
+      </c>
+      <c r="J52" s="6" t="inlineStr">
+        <is>
+          <t>Détail du compte (PBC, item 75)</t>
+        </is>
+      </c>
+      <c r="K52" s="6" t="inlineStr">
+        <is>
+          <t>Si le temps le permet</t>
+        </is>
+      </c>
+      <c r="L52" s="6" t="n"/>
+    </row>
+    <row r="53" ht="46" customHeight="1">
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Personnel</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Comment la provision pour départ à la retraite (compte 196) est-elle calculée ?</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>Provision reprise et dotée en totalité chaque année ; méthode inconnue.</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : barème de la convention collective, fichier du personnel, hypothèses.</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>Unités de crédit projetées</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>PIDR = Σ IDR × probabilité de présence × actualisation × prorata d'ancienneté</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>SYSCOHADA révisé ; convention collective interprofessionnelle</t>
+        </is>
+      </c>
+      <c r="J53" s="6" t="inlineStr">
+        <is>
+          <t>Note de calcul (PBC, items 76 à 78)</t>
+        </is>
+      </c>
+      <c r="K53" s="6" t="inlineStr">
+        <is>
+          <t>Si le temps le permet</t>
+        </is>
+      </c>
+      <c r="L53" s="6" t="n"/>
+    </row>
+    <row r="54" ht="46" customHeight="1">
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>Retraités</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>La garantie santé des retraités est-elle accordée à vie ?</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>Si oui, une provision mathématique est due.</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : règlement de la garantie.</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>Valeur actuelle des soins futurs</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>PM = Σ coût × probabilité de survie × actualisation</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>Règlement d'exécution n° 004/2022, art. 11</t>
+        </is>
+      </c>
+      <c r="J54" s="6" t="inlineStr">
+        <is>
+          <t>Règles de la garantie (PBC, item 79)</t>
+        </is>
+      </c>
+      <c r="K54" s="6" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L54" s="6" t="n"/>
+    </row>
+    <row r="55"/>
+    <row r="56">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Clôture de l'entretien</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="B50" s="18" t="inlineStr">
+    <row r="57">
+      <c r="B57" s="18" t="inlineStr">
         <is>
           <t>•  Récapituler les documents à obtenir : détail et fichiers de calcul des provisions 2019-2026, rapport actuariel existant, courriers de l'AIRMS, description de l'épargne et taux servis.</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="B51" s="18" t="inlineStr">
+    <row r="58">
+      <c r="B58" s="18" t="inlineStr">
         <is>
           <t>•  Demander : « Qui d'autre dois-je voir sur ces sujets ? »</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="B52" s="18" t="inlineStr">
+    <row r="59">
+      <c r="B59" s="18" t="inlineStr">
         <is>
           <t>•  Convenir d'une date de remise des documents et d'un contact pour les questions de suivi.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="B53" s="18" t="inlineStr">
+    <row r="60">
+      <c r="B60" s="18" t="inlineStr">
         <is>
           <t>•  Remercier l'interlocuteur.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="B4:L4"/>
     <mergeCell ref="B30:L30"/>
+    <mergeCell ref="B48:L48"/>
     <mergeCell ref="B33:L33"/>
     <mergeCell ref="B23:L23"/>
     <mergeCell ref="B5:L5"/>
@@ -4195,7 +4512,7 @@
     <mergeCell ref="B8:L8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="K8:K47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K8:K54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Entretiens placements et provisions du 19/10/2026 : comptes rendus, notes internes, PBC, guides, rapport v6
- Comptes rendus placements (14h) et provisions (16h) avec M. Koffi, chef comptable, logigrammes de la décision
  de placement et des allocations décès ; compte rendu cotisations complété (M. Kouamé Attuoman, participants)
- Notes internes confidentielles, une par entretien
- PBC complémentaire placements et provisions (items 80 à 99), reportée dans la PBC générale
- Guides : réponses et relances (placements, provisionnements), nom de l'interlocuteur cotisations
- Rapport v6 et classeur v6 : placements, méthode décès du FPPN, GNA apporteur d'affaires, compte 10620000,
  charges patronales de la provision retraite ; retouches de l'utilisateur sur la v5 reprises

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QrZoDwZJKb9thfUp96Ro9x
</commit_message>
<xml_diff>
--- a/FPPN_Guides_entretiens_actuariat_20261019.xlsx
+++ b/FPPN_Guides_entretiens_actuariat_20261019.xlsx
@@ -2477,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A2:L60"/>
+  <dimension ref="A2:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -4053,7 +4053,7 @@
       <c r="K45" s="15" t="n"/>
       <c r="L45" s="16" t="n"/>
     </row>
-    <row r="46" ht="46" customHeight="1">
+    <row r="46" ht="60" customHeight="1">
       <c r="B46" s="5" t="inlineStr">
         <is>
           <t>31</t>
@@ -4096,9 +4096,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L46" s="6" t="n"/>
-    </row>
-    <row r="47" ht="46" customHeight="1">
+      <c r="L46" s="6" t="inlineStr">
+        <is>
+          <t>Entretiens du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="60" customHeight="1">
       <c r="B47" s="5" t="inlineStr">
         <is>
           <t>32</t>
@@ -4145,7 +4149,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L47" s="6" t="n"/>
+      <c r="L47" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 16h avec M. Koffi (déclaration à confirmer par document) : 3,5 % pour la maladie et 1,5 % pour le décès, sans document qui fixe la répartition.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="B48" s="14" t="inlineStr">
@@ -4164,7 +4172,7 @@
       <c r="K48" s="15" t="n"/>
       <c r="L48" s="16" t="n"/>
     </row>
-    <row r="49" ht="46" customHeight="1">
+    <row r="49" ht="60" customHeight="1">
       <c r="B49" s="5" t="inlineStr">
         <is>
           <t>33</t>
@@ -4215,9 +4223,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L49" s="6" t="n"/>
-    </row>
-    <row r="50" ht="46" customHeight="1">
+      <c r="L49" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 16h avec M. Koffi (déclaration à confirmer par document) : montants hérités d'environ 2004, avant le PCMS ; jamais recalculés ; archives perdues lors d'un sinistre en 2010. Aucune provision maladie ; calcul de fin d'année des allocations décès restant à payer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="60" customHeight="1">
       <c r="B50" s="5" t="inlineStr">
         <is>
           <t>34</t>
@@ -4256,9 +4268,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L50" s="6" t="n"/>
-    </row>
-    <row r="51" ht="46" customHeight="1">
+      <c r="L50" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 16h avec M. Koffi (déclaration à confirmer par document) : les factures reçues jusqu'en mars sont rattachées à l'exercice (dettes) ; aucune provision maladie n'est calculée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="60" customHeight="1">
       <c r="B51" s="5" t="inlineStr">
         <is>
           <t>35</t>
@@ -4309,9 +4325,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L51" s="6" t="n"/>
-    </row>
-    <row r="52" ht="46" customHeight="1">
+      <c r="L51" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 16h avec M. Koffi (déclaration à confirmer par document) : le Grenier tient sa propre comptabilité de prêts ; la dépréciation n'a pas été abordée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="60" customHeight="1">
       <c r="B52" s="5" t="inlineStr">
         <is>
           <t>36</t>
@@ -4354,9 +4374,13 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L52" s="6" t="n"/>
-    </row>
-    <row r="53" ht="46" customHeight="1">
+      <c r="L52" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : le FPPN est apporteur d'affaires de GNA et perçoit 20 % des primes collectées, en fin d'année.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="60" customHeight="1">
       <c r="B53" s="5" t="inlineStr">
         <is>
           <t>37</t>
@@ -4407,9 +4431,13 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L53" s="6" t="n"/>
-    </row>
-    <row r="54" ht="46" customHeight="1">
+      <c r="L53" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 16h avec M. Koffi (déclaration à confirmer par document) : convention collective appliquée à l'ancienneté ; risques professionnels à 2 % ; fichiers de calcul et déclarations CNPS demandés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="60" customHeight="1">
       <c r="B54" s="5" t="inlineStr">
         <is>
           <t>38</t>
@@ -4460,50 +4488,207 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L54" s="6" t="n"/>
-    </row>
-    <row r="55"/>
-    <row r="56">
-      <c r="B56" s="2" t="inlineStr">
+      <c r="L54" s="6" t="inlineStr">
+        <is>
+          <t>Entretiens du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>J. Relances après l'entretien du 19/10/2026 (16h)</t>
+        </is>
+      </c>
+      <c r="C55" s="15" t="n"/>
+      <c r="D55" s="15" t="n"/>
+      <c r="E55" s="15" t="n"/>
+      <c r="F55" s="15" t="n"/>
+      <c r="G55" s="15" t="n"/>
+      <c r="H55" s="15" t="n"/>
+      <c r="I55" s="15" t="n"/>
+      <c r="J55" s="15" t="n"/>
+      <c r="K55" s="15" t="n"/>
+      <c r="L55" s="16" t="n"/>
+    </row>
+    <row r="56" ht="46" customHeight="1">
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>Décès</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>Dans quel compte le calcul de fin d'année des allocations décès restant à payer est-il comptabilisé ?</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>Le compte 15802000 ne bouge pas depuis 2020.</t>
+        </is>
+      </c>
+      <c r="F56" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : compte et calculs 2020 à 2025.</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="n"/>
+      <c r="H56" s="6" t="n"/>
+      <c r="I56" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J56" s="6" t="inlineStr">
+        <is>
+          <t>PBC, item 92</t>
+        </is>
+      </c>
+      <c r="K56" s="6" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L56" s="6" t="n"/>
+    </row>
+    <row r="57" ht="46" customHeight="1">
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Décès</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Quel est le montant de l'allocation décès d'un officier ?</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="inlineStr">
+        <is>
+          <t>Montant non lisible dans la transcription.</t>
+        </is>
+      </c>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : barème officiel.</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="n"/>
+      <c r="H57" s="6" t="n"/>
+      <c r="I57" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J57" s="6" t="inlineStr">
+        <is>
+          <t>PBC, item 93</t>
+        </is>
+      </c>
+      <c r="K57" s="6" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L57" s="6" t="n"/>
+    </row>
+    <row r="58" ht="46" customHeight="1">
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>Provisions</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>Quand et par quel courrier l'AIRMS a-t-elle demandé le reclassement des provisions en compte 158 ?</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>Le reclassement est visible dans la balance 2024.</t>
+        </is>
+      </c>
+      <c r="F58" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : courrier de l'AIRMS.</t>
+        </is>
+      </c>
+      <c r="G58" s="6" t="n"/>
+      <c r="H58" s="6" t="n"/>
+      <c r="I58" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J58" s="6" t="inlineStr">
+        <is>
+          <t>PBC, item 95</t>
+        </is>
+      </c>
+      <c r="K58" s="6" t="inlineStr">
+        <is>
+          <t>Si le temps le permet</t>
+        </is>
+      </c>
+      <c r="L58" s="6" t="n"/>
+    </row>
+    <row r="59"/>
+    <row r="60">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>Clôture de l'entretien</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="B57" s="18" t="inlineStr">
+    <row r="61">
+      <c r="B61" s="18" t="inlineStr">
         <is>
           <t>•  Récapituler les documents à obtenir : détail et fichiers de calcul des provisions 2019-2026, rapport actuariel existant, courriers de l'AIRMS, description de l'épargne et taux servis.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="B58" s="18" t="inlineStr">
+    <row r="62">
+      <c r="B62" s="18" t="inlineStr">
         <is>
           <t>•  Demander : « Qui d'autre dois-je voir sur ces sujets ? »</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="B59" s="18" t="inlineStr">
+    <row r="63">
+      <c r="B63" s="18" t="inlineStr">
         <is>
           <t>•  Convenir d'une date de remise des documents et d'un contact pour les questions de suivi.</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="B60" s="18" t="inlineStr">
+    <row r="64">
+      <c r="B64" s="18" t="inlineStr">
         <is>
           <t>•  Remercier l'interlocuteur.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="B4:L4"/>
     <mergeCell ref="B30:L30"/>
     <mergeCell ref="B48:L48"/>
     <mergeCell ref="B33:L33"/>
+    <mergeCell ref="B55:L55"/>
     <mergeCell ref="B23:L23"/>
     <mergeCell ref="B5:L5"/>
     <mergeCell ref="B45:L45"/>
@@ -4512,7 +4697,7 @@
     <mergeCell ref="B8:L8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="K8:K54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K8:K58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4528,7 +4713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:L37"/>
+  <dimension ref="A2:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -4555,7 +4740,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>16 octobre 2026, 14h, avec Marlène Mody</t>
+          <t>16 octobre 2026, 14h, avec Marlène Mody ; entretien tenu le 19/10/2026 à 14h avec M. Koffi, chef comptable</t>
         </is>
       </c>
     </row>
@@ -4684,9 +4869,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="46" customHeight="1">
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : DAT BOA alimenté chaque mois (60 millions par mois en 2026) et débouclé en fin d'année ; FCP de 500 millions géré par United Capital (SGI) ; terrains. Aucune obligation ni action citée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
       <c r="B10" s="5" t="n">
         <v>2</v>
       </c>
@@ -4731,9 +4920,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L10" s="6" t="inlineStr"/>
-    </row>
-    <row r="11" ht="46" customHeight="1">
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : BOA pour le DAT, United Capital (SGI) pour le FCP ; Orabank par le passé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
       <c r="B11" s="5" t="n">
         <v>3</v>
       </c>
@@ -4778,9 +4971,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L11" s="6" t="inlineStr"/>
-    </row>
-    <row r="12" ht="46" customHeight="1">
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : le DAT court jusqu'au 30 ou 31 décembre ; pas d'échéance citée pour le FCP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
       <c r="B12" s="5" t="n">
         <v>4</v>
       </c>
@@ -4821,9 +5018,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13" ht="46" customHeight="1">
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>Entretiens du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
       <c r="B13" s="5" t="n">
         <v>5</v>
       </c>
@@ -4864,7 +5065,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr"/>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : FCP : rendement annoncé de 8 à 10 %, non garanti. Taux du DAT non communiqué.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="14" t="inlineStr">
@@ -4883,7 +5088,7 @@
       <c r="K14" s="15" t="n"/>
       <c r="L14" s="16" t="n"/>
     </row>
-    <row r="15" ht="46" customHeight="1">
+    <row r="15" ht="60" customHeight="1">
       <c r="B15" s="5" t="n">
         <v>6</v>
       </c>
@@ -4924,7 +5129,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : aucune politique écrite ; toutes les décisions viennent de la direction générale ; ni comité ni avis du conseil d'administration.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="B16" s="5" t="n">
@@ -4971,9 +5180,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr"/>
-    </row>
-    <row r="17" ht="46" customHeight="1">
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : le montant du DAT est fixé selon les départs à la retraite prévus (liste de la direction du personnel) et une simulation de la comptabilité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1">
       <c r="B17" s="5" t="n">
         <v>8</v>
       </c>
@@ -5010,7 +5223,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr"/>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>Entretiens du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="B18" s="14" t="inlineStr">
@@ -5029,7 +5246,7 @@
       <c r="K18" s="15" t="n"/>
       <c r="L18" s="16" t="n"/>
     </row>
-    <row r="19" ht="46" customHeight="1">
+    <row r="19" ht="60" customHeight="1">
       <c r="B19" s="5" t="n">
         <v>9</v>
       </c>
@@ -5074,9 +5291,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20" ht="46" customHeight="1">
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : liste des départs à la retraite fournie par la direction du personnel, rapprochée des souscripteurs, puis simulation par la comptabilité.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1">
       <c r="B20" s="5" t="n">
         <v>10</v>
       </c>
@@ -5109,7 +5330,11 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L20" s="6" t="inlineStr"/>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>Entretiens du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="14" t="inlineStr">
@@ -5128,7 +5353,7 @@
       <c r="K21" s="15" t="n"/>
       <c r="L21" s="16" t="n"/>
     </row>
-    <row r="22" ht="46" customHeight="1">
+    <row r="22" ht="60" customHeight="1">
       <c r="B22" s="5" t="n">
         <v>11</v>
       </c>
@@ -5177,9 +5402,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23" ht="46" customHeight="1">
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : le Trésor vire parfois partiellement ; le reste est versé plus tard ; le DAF relance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1">
       <c r="B23" s="5" t="n">
         <v>12</v>
       </c>
@@ -5228,9 +5457,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L23" s="6" t="inlineStr"/>
-    </row>
-    <row r="24" ht="32" customHeight="1">
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : le Grenier tient sa propre comptabilité de prêts dans un logiciel de microfinance ; impayés non abordés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1">
       <c r="B24" s="5" t="n">
         <v>13</v>
       </c>
@@ -5275,9 +5508,13 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25" ht="46" customHeight="1">
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : le terrain du siège a été réévalué par un expert immobilier (compte 10620000) ; date non précisée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1">
       <c r="B25" s="5" t="n">
         <v>14</v>
       </c>
@@ -5310,7 +5547,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L25" s="6" t="inlineStr"/>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : deux villas et un autre bâtiment à Aboisso sont loués à usage d'habitation ; pas de programme de location-vente cité.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="14" t="inlineStr">
@@ -5329,7 +5570,7 @@
       <c r="K26" s="15" t="n"/>
       <c r="L26" s="16" t="n"/>
     </row>
-    <row r="27" ht="32" customHeight="1">
+    <row r="27" ht="60" customHeight="1">
       <c r="B27" s="5" t="n">
         <v>15</v>
       </c>
@@ -5362,9 +5603,13 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L27" s="6" t="inlineStr"/>
-    </row>
-    <row r="28" ht="46" customHeight="1">
+      <c r="L27" s="6" t="inlineStr">
+        <is>
+          <t>Entretiens du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="60" customHeight="1">
       <c r="B28" s="5" t="n">
         <v>16</v>
       </c>
@@ -5397,7 +5642,11 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L28" s="6" t="inlineStr"/>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : les placements sont suivis sur les relevés bancaires ; les rapprochements bancaires ne sont plus supervisés.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="B29" s="14" t="inlineStr">
@@ -5416,7 +5665,7 @@
       <c r="K29" s="15" t="n"/>
       <c r="L29" s="16" t="n"/>
     </row>
-    <row r="30" ht="46" customHeight="1">
+    <row r="30" ht="60" customHeight="1">
       <c r="B30" s="5" t="n">
         <v>17</v>
       </c>
@@ -5457,9 +5706,13 @@
           <t>Incontournable</t>
         </is>
       </c>
-      <c r="L30" s="6" t="inlineStr"/>
-    </row>
-    <row r="31" ht="46" customHeight="1">
+      <c r="L30" s="6" t="inlineStr">
+        <is>
+          <t>Entretiens du 19/10/2026 : pas de réponse relevée sur ce point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="60" customHeight="1">
       <c r="B31" s="5" t="n">
         <v>18</v>
       </c>
@@ -5500,60 +5753,361 @@
           <t>Si le temps le permet</t>
         </is>
       </c>
-      <c r="L31" s="6" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="B33" s="2" t="inlineStr">
+      <c r="L31" s="6" t="inlineStr">
+        <is>
+          <t>Entretien du 19/10/2026 à 14h avec M. Koffi (déclaration à confirmer par document) : aucun placement bloqué cité ; incident passé avec Orabank (versements arrêtés, DAT remboursé au terme).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>G. Relances après l'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="C32" s="15" t="n"/>
+      <c r="D32" s="15" t="n"/>
+      <c r="E32" s="15" t="n"/>
+      <c r="F32" s="15" t="n"/>
+      <c r="G32" s="15" t="n"/>
+      <c r="H32" s="15" t="n"/>
+      <c r="I32" s="15" t="n"/>
+      <c r="J32" s="15" t="n"/>
+      <c r="K32" s="15" t="n"/>
+      <c r="L32" s="16" t="n"/>
+    </row>
+    <row r="33" ht="46" customHeight="1">
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>DAT</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Quel est le taux du DAT BOA, et pourquoi le compte 52210200 s'intitule-t-il « Entraide fin de carrière » ?</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Confirmer la nature et le rendement du principal placement.</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : convention et relevés.</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="n"/>
+      <c r="H33" s="6" t="n"/>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>PBC, item 80</t>
+        </is>
+      </c>
+      <c r="K33" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L33" s="6" t="n"/>
+    </row>
+    <row r="34" ht="46" customHeight="1">
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>FCP</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Quelle est la valeur liquidative du FCP au 31/08/2026 et son rendement réel depuis la souscription ?</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Le FCP n'est pas revalorisé dans les comptes.</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : relevés du gestionnaire.</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="n"/>
+      <c r="H34" s="6" t="inlineStr">
+        <is>
+          <t>Rendement = (valeur finale - valeur initiale) / valeur initiale</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J34" s="6" t="inlineStr">
+        <is>
+          <t>PBC, item 81</t>
+        </is>
+      </c>
+      <c r="K34" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L34" s="6" t="n"/>
+    </row>
+    <row r="35" ht="46" customHeight="1">
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Orabank</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>En quelle année l'incident Orabank a-t-il eu lieu ? Les balances montrent un DAT ouvert en 2022 et soldé en 2023.</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Dater l'incident cité.</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : correspondance avec la banque.</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="n"/>
+      <c r="H35" s="6" t="n"/>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>PBC, item 83</t>
+        </is>
+      </c>
+      <c r="K35" s="17" t="inlineStr">
+        <is>
+          <t>Si le temps le permet</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="n"/>
+    </row>
+    <row r="36" ht="46" customHeight="1">
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>GNA</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Sur quelle assiette la commission de 20 % est-elle calculée ? En 2024, la commission comptabilisée ne vaut pas 20 % des précomptes 9W3.</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Rapprocher les commissions des primes.</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : convention et décomptes.</t>
+        </is>
+      </c>
+      <c r="G36" s="6" t="n"/>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>Commission = 20 % × primes collectées</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>PBC, item 89</t>
+        </is>
+      </c>
+      <c r="K36" s="17" t="inlineStr">
+        <is>
+          <t>Si le temps le permet</t>
+        </is>
+      </c>
+      <c r="L36" s="6" t="n"/>
+    </row>
+    <row r="37" ht="46" customHeight="1">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Terrains</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Quels sont les terrains du FPPN, leur situation et les projets prévus ?</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Évaluer les actifs immobiliers.</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : inventaire et titres.</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="n"/>
+      <c r="H37" s="6" t="n"/>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>PBC, item 84</t>
+        </is>
+      </c>
+      <c r="K37" s="17" t="inlineStr">
+        <is>
+          <t>Si le temps le permet</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="n"/>
+    </row>
+    <row r="38" ht="46" customHeight="1">
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Hôpital</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Où en sont les démarches auprès de l'État sur la créance de l'hôpital de la Police ?</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Apprécier le recouvrement de 3 407 519 850 FCFA.</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>Attendu : correspondances et décision.</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="n"/>
+      <c r="H38" s="6" t="n"/>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>Compte rendu d'entretien du 19/10/2026</t>
+        </is>
+      </c>
+      <c r="J38" s="6" t="inlineStr">
+        <is>
+          <t>PBC, item 87</t>
+        </is>
+      </c>
+      <c r="K38" s="17" t="inlineStr">
+        <is>
+          <t>Incontournable</t>
+        </is>
+      </c>
+      <c r="L38" s="6" t="n"/>
+    </row>
+    <row r="39"/>
+    <row r="40">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Clôture de l'entretien</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="B34" s="18" t="inlineStr">
+    <row r="41" ht="30" customHeight="1">
+      <c r="B41" s="18" t="inlineStr">
         <is>
           <t>•  Récapituler les documents à obtenir : inventaire et échéancier des placements, politique de placement, prévisions de trésorerie, état des cotisations non reversées, encours des prêts.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="B35" s="18" t="inlineStr">
+    <row r="42" ht="16" customHeight="1">
+      <c r="B42" s="18" t="inlineStr">
         <is>
           <t>•  Demander : « Qui d'autre dois-je voir sur ces sujets ? »</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="B36" s="18" t="inlineStr">
+    <row r="43" ht="16" customHeight="1">
+      <c r="B43" s="18" t="inlineStr">
         <is>
           <t>•  Convenir d'une date de remise des documents et d'un contact pour les questions de suivi.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="B37" s="18" t="inlineStr">
+    <row r="44" ht="16" customHeight="1">
+      <c r="B44" s="18" t="inlineStr">
         <is>
           <t>•  Remercier l'interlocuteur.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="B35:L35"/>
+  <mergeCells count="13">
     <mergeCell ref="B4:L4"/>
     <mergeCell ref="B26:L26"/>
+    <mergeCell ref="B43:L43"/>
+    <mergeCell ref="B41:L41"/>
     <mergeCell ref="B21:L21"/>
+    <mergeCell ref="B44:L44"/>
     <mergeCell ref="B29:L29"/>
     <mergeCell ref="B5:L5"/>
-    <mergeCell ref="B34:L34"/>
-    <mergeCell ref="B37:L37"/>
-    <mergeCell ref="B36:L36"/>
+    <mergeCell ref="B42:L42"/>
     <mergeCell ref="B14:L14"/>
+    <mergeCell ref="B32:L32"/>
     <mergeCell ref="B18:L18"/>
     <mergeCell ref="B8:L8"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="K8:K32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K8:K38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Incontournable,Si le temps le permet"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5596,7 +6150,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>19 octobre 2026, 10h, avec Ruth Miensa ; entretien tenu avec le responsable des cotisations, également responsable informatique (nom à compléter)</t>
+          <t>19 octobre 2026, 10h, avec Ruth Miensa ; entretien tenu avec le responsable des cotisations, également responsable informatique (M. Kouamé Attuoman)</t>
         </is>
       </c>
     </row>

</xml_diff>